<commit_message>
chore: track updated sample fixture, ignore Excel lock files
</commit_message>
<xml_diff>
--- a/fixtures/mahasiswa-sample.xlsx
+++ b/fixtures/mahasiswa-sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\002. NGULIah\003. CODESOURCES\project0\traffic_tracker\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314A0970-B3F3-4303-81A4-C91839907D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49169F5F-DB63-4B1A-9032-BDEAA578B9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
   <si>
     <t>NIM</t>
   </si>
@@ -34,9 +34,6 @@
     <t>KELAS</t>
   </si>
   <si>
-    <t>4420231001</t>
-  </si>
-  <si>
     <t>BUDI SANTOSO</t>
   </si>
   <si>
@@ -140,6 +137,12 @@
   </si>
   <si>
     <t>RUDI HARTONO</t>
+  </si>
+  <si>
+    <t>Galang ji Won</t>
+  </si>
+  <si>
+    <t>A2</t>
   </si>
 </sst>
 </file>
@@ -175,8 +178,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -516,16 +522,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.59765625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.69921875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -539,248 +545,262 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>4420231001</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
       </c>
       <c r="C2">
         <v>3</v>
       </c>
       <c r="D2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
       </c>
       <c r="C3">
         <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
         <v>10</v>
       </c>
-      <c r="C4">
-        <v>5</v>
-      </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>13</v>
       </c>
-      <c r="C5">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
         <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
         <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>18</v>
       </c>
       <c r="C7">
         <v>7</v>
       </c>
       <c r="D7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>4420231004</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8">
         <v>3</v>
       </c>
       <c r="D8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
         <v>20</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>21</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>22</v>
       </c>
-      <c r="D9" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>24</v>
-      </c>
-      <c r="B10" t="s">
-        <v>25</v>
       </c>
       <c r="C10">
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" t="s">
         <v>26</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>27</v>
       </c>
-      <c r="C11">
-        <v>5</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
         <v>28</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12">
+        <v>5</v>
+      </c>
+      <c r="D12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>29</v>
       </c>
-      <c r="C12">
-        <v>5</v>
-      </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
         <v>30</v>
-      </c>
-      <c r="B13" t="s">
-        <v>31</v>
       </c>
       <c r="C13">
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" t="s">
         <v>32</v>
-      </c>
-      <c r="B14" t="s">
-        <v>33</v>
       </c>
       <c r="C14">
         <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C15">
         <v>3</v>
       </c>
       <c r="D15" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" t="s">
         <v>35</v>
-      </c>
-      <c r="B16" t="s">
-        <v>36</v>
       </c>
       <c r="C16">
         <v>3</v>
       </c>
       <c r="D16" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C17">
         <v>3</v>
       </c>
       <c r="D17" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" t="s">
         <v>38</v>
-      </c>
-      <c r="B18" t="s">
-        <v>39</v>
       </c>
       <c r="C18">
         <v>1</v>
       </c>
       <c r="D18" t="s">
-        <v>16</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>462025611059</v>
+      </c>
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19">
+        <v>14</v>
+      </c>
+      <c r="D19" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D18" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D1 A3:D18 B2:D2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>